<commit_message>
Fix mistyped 80*40 sale as 80*60 in label master and report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qcxxm45opVsMXpkD7SANqh
</commit_message>
<xml_diff>
--- a/라벨 마스터 V16.xlsx
+++ b/라벨 마스터 V16.xlsx
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="195">
   <si>
     <t xml:space="preserve">라벨 마스터 (재질·규격별 입고/출고/재고·가격·채널별 판매) — 재고 2026-10-07 실재고 · 오픈마켓 판매는 판매현황 시트 기준</t>
   </si>
@@ -1457,9 +1457,6 @@
   </si>
   <si>
     <t xml:space="preserve">품절/재고없음</t>
-  </si>
-  <si>
-    <t xml:space="preserve">80*40</t>
   </si>
   <si>
     <t xml:space="preserve">코스모스몰</t>
@@ -3937,18 +3934,18 @@
       </c>
       <c r="F11" s="13" t="n">
         <f aca="false">S11+T11+U11+V11+Z11</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G11" s="12" t="n">
         <v>13</v>
       </c>
       <c r="H11" s="14" t="n">
         <f aca="false">COUNTIFS(판매현황!$C$3:$C$1000,LEFT($B11,3),판매현황!$D$3:$D$1000,$C11,판매현황!$G$3:$G$1000,"&gt;0")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11" s="15" t="n">
         <f aca="false">IF(E11=0,"",F11/E11)</f>
-        <v>0.0229885057471264</v>
+        <v>0.0344827586206897</v>
       </c>
       <c r="J11" s="16" t="n">
         <f aca="false">COUNTIFS($A$5:$A$30,"&gt;0",$G$5:$G$30,"&gt;"&amp;G11)+1</f>
@@ -3993,7 +3990,7 @@
       </c>
       <c r="U11" s="13" t="n">
         <f aca="false">SUMIFS(판매현황!$G$3:$G$1000,판매현황!$C$3:$C$1000,LEFT($B11,3),판매현황!$D$3:$D$1000,$C11,판매현황!$F$3:$F$1000,"전문몰")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V11" s="13" t="n">
         <f aca="false">SUMIFS(판매현황!$G$3:$G$1000,판매현황!$C$3:$C$1000,LEFT($B11,3),판매현황!$D$3:$D$1000,$C11,판매현황!$F$3:$F$1000,"11번가")</f>
@@ -4016,7 +4013,7 @@
       </c>
       <c r="AA11" s="13" t="n">
         <f aca="false">E11-F11</f>
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4338,7 +4335,7 @@
       </c>
       <c r="F15" s="26" t="n">
         <f aca="false">SUM(F5:F14)</f>
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G15" s="26" t="n">
         <f aca="false">SUM(G5:G14)</f>
@@ -4346,7 +4343,7 @@
       </c>
       <c r="H15" s="26" t="n">
         <f aca="false">SUM(H5:H14)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I15" s="27"/>
       <c r="J15" s="27"/>
@@ -4368,7 +4365,7 @@
       </c>
       <c r="U15" s="26" t="n">
         <f aca="false">SUM(U5:U14)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="V15" s="26" t="n">
         <f aca="false">SUM(V5:V14)</f>
@@ -4383,7 +4380,7 @@
       </c>
       <c r="AA15" s="26" t="n">
         <f aca="false">SUM(AA5:AA14)</f>
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5941,7 +5938,7 @@
       </c>
       <c r="F32" s="33" t="n">
         <f aca="false">F15+F28+F31</f>
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G32" s="33" t="n">
         <f aca="false">G15+G28+G31</f>
@@ -5949,7 +5946,7 @@
       </c>
       <c r="H32" s="33" t="n">
         <f aca="false">H15+H28+H31</f>
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I32" s="34"/>
       <c r="J32" s="34"/>
@@ -5971,7 +5968,7 @@
       </c>
       <c r="U32" s="33" t="n">
         <f aca="false">U15+U28+U31</f>
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="V32" s="33" t="n">
         <f aca="false">V15+V28+V31</f>
@@ -5986,7 +5983,7 @@
       </c>
       <c r="AA32" s="33" t="n">
         <f aca="false">AA15+AA28+AA31</f>
-        <v>776</v>
+        <v>775</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6313,7 +6310,7 @@
       </c>
       <c r="G44" s="20" t="n">
         <f aca="false">U11</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H44" s="20" t="n">
         <f aca="false">Z11</f>
@@ -6977,7 +6974,7 @@
       </c>
       <c r="C62" s="46" t="n">
         <f aca="false">D62+E62+F62+G62+H62</f>
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D62" s="46" t="n">
         <f aca="false">SUM(D38:D61)</f>
@@ -6993,7 +6990,7 @@
       </c>
       <c r="G62" s="46" t="n">
         <f aca="false">SUM(G38:G61)</f>
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H62" s="46" t="n">
         <f aca="false">SUM(H38:H61)</f>
@@ -7369,11 +7366,11 @@
       </c>
       <c r="E10" s="54" t="n">
         <f aca="false">마스터!F11</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" s="54" t="n">
         <f aca="false">마스터!E11-마스터!F11</f>
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G10" s="54" t="n">
         <f aca="false">IF(ISBLANK(마스터!O11),"미기재",마스터!O11)</f>
@@ -7532,11 +7529,11 @@
       </c>
       <c r="E14" s="67" t="n">
         <f aca="false">SUM(E4:E13)</f>
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F14" s="67" t="n">
         <f aca="false">SUM(F4:F13)</f>
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="G14" s="68"/>
       <c r="H14" s="68"/>
@@ -13493,7 +13490,7 @@
         <v>30</v>
       </c>
       <c r="D39" s="140" t="s">
-        <v>194</v>
+        <v>43</v>
       </c>
       <c r="E39" s="141"/>
       <c r="F39" s="139" t="s">
@@ -13805,7 +13802,7 @@
       </c>
       <c r="E53" s="141"/>
       <c r="F53" s="139" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G53" s="149" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
Remove non-China-label 80*40 sale record
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qcxxm45opVsMXpkD7SANqh
</commit_message>
<xml_diff>
--- a/라벨 마스터 V16.xlsx
+++ b/라벨 마스터 V16.xlsx
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="195">
   <si>
     <t xml:space="preserve">라벨 마스터 (재질·규격별 입고/출고/재고·가격·채널별 판매) — 재고 2026-10-07 실재고 · 오픈마켓 판매는 판매현황 시트 기준</t>
   </si>
@@ -3934,18 +3934,18 @@
       </c>
       <c r="F11" s="13" t="n">
         <f aca="false">S11+T11+U11+V11+Z11</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11" s="12" t="n">
         <v>13</v>
       </c>
       <c r="H11" s="14" t="n">
         <f aca="false">COUNTIFS(판매현황!$C$3:$C$1000,LEFT($B11,3),판매현황!$D$3:$D$1000,$C11,판매현황!$G$3:$G$1000,"&gt;0")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I11" s="15" t="n">
         <f aca="false">IF(E11=0,"",F11/E11)</f>
-        <v>0.0344827586206897</v>
+        <v>0.0229885057471264</v>
       </c>
       <c r="J11" s="16" t="n">
         <f aca="false">COUNTIFS($A$5:$A$30,"&gt;0",$G$5:$G$30,"&gt;"&amp;G11)+1</f>
@@ -3990,7 +3990,7 @@
       </c>
       <c r="U11" s="13" t="n">
         <f aca="false">SUMIFS(판매현황!$G$3:$G$1000,판매현황!$C$3:$C$1000,LEFT($B11,3),판매현황!$D$3:$D$1000,$C11,판매현황!$F$3:$F$1000,"전문몰")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V11" s="13" t="n">
         <f aca="false">SUMIFS(판매현황!$G$3:$G$1000,판매현황!$C$3:$C$1000,LEFT($B11,3),판매현황!$D$3:$D$1000,$C11,판매현황!$F$3:$F$1000,"11번가")</f>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="AA11" s="13" t="n">
         <f aca="false">E11-F11</f>
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="F15" s="26" t="n">
         <f aca="false">SUM(F5:F14)</f>
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G15" s="26" t="n">
         <f aca="false">SUM(G5:G14)</f>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="H15" s="26" t="n">
         <f aca="false">SUM(H5:H14)</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I15" s="27"/>
       <c r="J15" s="27"/>
@@ -4365,7 +4365,7 @@
       </c>
       <c r="U15" s="26" t="n">
         <f aca="false">SUM(U5:U14)</f>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="V15" s="26" t="n">
         <f aca="false">SUM(V5:V14)</f>
@@ -4380,7 +4380,7 @@
       </c>
       <c r="AA15" s="26" t="n">
         <f aca="false">SUM(AA5:AA14)</f>
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5938,7 +5938,7 @@
       </c>
       <c r="F32" s="33" t="n">
         <f aca="false">F15+F28+F31</f>
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G32" s="33" t="n">
         <f aca="false">G15+G28+G31</f>
@@ -5946,7 +5946,7 @@
       </c>
       <c r="H32" s="33" t="n">
         <f aca="false">H15+H28+H31</f>
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I32" s="34"/>
       <c r="J32" s="34"/>
@@ -5968,7 +5968,7 @@
       </c>
       <c r="U32" s="33" t="n">
         <f aca="false">U15+U28+U31</f>
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="V32" s="33" t="n">
         <f aca="false">V15+V28+V31</f>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="AA32" s="33" t="n">
         <f aca="false">AA15+AA28+AA31</f>
-        <v>775</v>
+        <v>776</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="G44" s="20" t="n">
         <f aca="false">U11</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H44" s="20" t="n">
         <f aca="false">Z11</f>
@@ -6974,7 +6974,7 @@
       </c>
       <c r="C62" s="46" t="n">
         <f aca="false">D62+E62+F62+G62+H62</f>
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D62" s="46" t="n">
         <f aca="false">SUM(D38:D61)</f>
@@ -6990,7 +6990,7 @@
       </c>
       <c r="G62" s="46" t="n">
         <f aca="false">SUM(G38:G61)</f>
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H62" s="46" t="n">
         <f aca="false">SUM(H38:H61)</f>
@@ -7366,11 +7366,11 @@
       </c>
       <c r="E10" s="54" t="n">
         <f aca="false">마스터!F11</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" s="54" t="n">
         <f aca="false">마스터!E11-마스터!F11</f>
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G10" s="54" t="n">
         <f aca="false">IF(ISBLANK(마스터!O11),"미기재",마스터!O11)</f>
@@ -7529,11 +7529,11 @@
       </c>
       <c r="E14" s="67" t="n">
         <f aca="false">SUM(E4:E13)</f>
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F14" s="67" t="n">
         <f aca="false">SUM(F4:F13)</f>
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G14" s="68"/>
       <c r="H14" s="68"/>
@@ -13484,20 +13484,20 @@
         <v>46119</v>
       </c>
       <c r="B39" s="138" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="C39" s="139" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D39" s="140" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="E39" s="141"/>
       <c r="F39" s="139" t="s">
         <v>80</v>
       </c>
       <c r="G39" s="149" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H39" s="140"/>
     </row>
@@ -13512,14 +13512,14 @@
         <v>50</v>
       </c>
       <c r="D40" s="140" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E40" s="141"/>
       <c r="F40" s="139" t="s">
         <v>80</v>
       </c>
       <c r="G40" s="149" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H40" s="140"/>
     </row>
@@ -13528,13 +13528,13 @@
         <v>46119</v>
       </c>
       <c r="B41" s="138" t="n">
-        <v>46269</v>
+        <v>46275</v>
       </c>
       <c r="C41" s="139" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="D41" s="140" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="E41" s="141"/>
       <c r="F41" s="139" t="s">
@@ -13550,20 +13550,20 @@
         <v>46119</v>
       </c>
       <c r="B42" s="138" t="n">
-        <v>46275</v>
+        <v>46286</v>
       </c>
       <c r="C42" s="139" t="s">
         <v>30</v>
       </c>
-      <c r="D42" s="140" t="s">
-        <v>43</v>
+      <c r="D42" s="145" t="s">
+        <v>39</v>
       </c>
       <c r="E42" s="141"/>
       <c r="F42" s="139" t="s">
         <v>80</v>
       </c>
       <c r="G42" s="149" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H42" s="140"/>
     </row>
@@ -13572,13 +13572,13 @@
         <v>46119</v>
       </c>
       <c r="B43" s="138" t="n">
-        <v>46286</v>
+        <v>46295</v>
       </c>
       <c r="C43" s="139" t="s">
-        <v>30</v>
-      </c>
-      <c r="D43" s="145" t="s">
-        <v>39</v>
+        <v>50</v>
+      </c>
+      <c r="D43" s="140" t="s">
+        <v>56</v>
       </c>
       <c r="E43" s="141"/>
       <c r="F43" s="139" t="s">
@@ -13600,14 +13600,14 @@
         <v>50</v>
       </c>
       <c r="D44" s="140" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="E44" s="141"/>
       <c r="F44" s="139" t="s">
         <v>80</v>
       </c>
       <c r="G44" s="149" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H44" s="140"/>
     </row>
@@ -13619,14 +13619,14 @@
         <v>46295</v>
       </c>
       <c r="C45" s="139" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="D45" s="140" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E45" s="141"/>
       <c r="F45" s="139" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G45" s="149" t="n">
         <v>1</v>
@@ -13641,14 +13641,14 @@
         <v>46295</v>
       </c>
       <c r="C46" s="139" t="s">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="D46" s="140" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E46" s="141"/>
       <c r="F46" s="139" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G46" s="149" t="n">
         <v>1</v>
@@ -13660,20 +13660,20 @@
         <v>46119</v>
       </c>
       <c r="B47" s="138" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="C47" s="139" t="s">
         <v>30</v>
       </c>
       <c r="D47" s="140" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="E47" s="141"/>
       <c r="F47" s="139" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="G47" s="149" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H47" s="140"/>
     </row>
@@ -13682,20 +13682,20 @@
         <v>46119</v>
       </c>
       <c r="B48" s="138" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="C48" s="139" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D48" s="140" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="E48" s="141"/>
       <c r="F48" s="139" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G48" s="149" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H48" s="140"/>
     </row>
@@ -13704,17 +13704,17 @@
         <v>46119</v>
       </c>
       <c r="B49" s="138" t="n">
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="C49" s="139" t="s">
-        <v>50</v>
-      </c>
-      <c r="D49" s="140" t="s">
-        <v>51</v>
+        <v>30</v>
+      </c>
+      <c r="D49" s="145" t="s">
+        <v>39</v>
       </c>
       <c r="E49" s="141"/>
       <c r="F49" s="139" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="G49" s="149" t="n">
         <v>1</v>
@@ -13751,17 +13751,17 @@
         <v>46301</v>
       </c>
       <c r="C51" s="139" t="s">
-        <v>30</v>
-      </c>
-      <c r="D51" s="145" t="s">
-        <v>39</v>
+        <v>68</v>
+      </c>
+      <c r="D51" s="140" t="s">
+        <v>69</v>
       </c>
       <c r="E51" s="141"/>
       <c r="F51" s="139" t="s">
         <v>77</v>
       </c>
       <c r="G51" s="149" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H51" s="140"/>
     </row>
@@ -13776,37 +13776,25 @@
         <v>68</v>
       </c>
       <c r="D52" s="140" t="s">
-        <v>69</v>
+        <v>47</v>
       </c>
       <c r="E52" s="141"/>
       <c r="F52" s="139" t="s">
-        <v>77</v>
+        <v>194</v>
       </c>
       <c r="G52" s="149" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H52" s="140"/>
     </row>
     <row r="53" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="137" t="n">
-        <v>46119</v>
-      </c>
-      <c r="B53" s="138" t="n">
-        <v>46301</v>
-      </c>
-      <c r="C53" s="139" t="s">
-        <v>68</v>
-      </c>
-      <c r="D53" s="140" t="s">
-        <v>47</v>
-      </c>
+      <c r="A53" s="137"/>
+      <c r="B53" s="138"/>
+      <c r="C53" s="139"/>
+      <c r="D53" s="140"/>
       <c r="E53" s="141"/>
-      <c r="F53" s="139" t="s">
-        <v>194</v>
-      </c>
-      <c r="G53" s="149" t="n">
-        <v>6</v>
-      </c>
+      <c r="F53" s="139"/>
+      <c r="G53" s="149"/>
       <c r="H53" s="140"/>
     </row>
     <row r="54" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13830,36 +13818,27 @@
       <c r="H55" s="140"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="137"/>
-      <c r="B56" s="138"/>
-      <c r="C56" s="139"/>
-      <c r="D56" s="140"/>
-      <c r="E56" s="141"/>
-      <c r="F56" s="139"/>
-      <c r="G56" s="149"/>
-      <c r="H56" s="140"/>
+      <c r="H56" s="145"/>
     </row>
     <row r="57" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H57" s="145"/>
+      <c r="G57" s="131" t="n">
+        <f aca="false">SUBTOTAL(9,G3:G55)</f>
+        <v>228</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="G58" s="131" t="n">
-        <f aca="false">SUBTOTAL(9,G3:G56)</f>
-        <v>229</v>
-      </c>
+      <c r="G58" s="167"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G59" s="167"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="G60" s="167"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="G61" s="131" t="n">
-        <f aca="false">SUBTOTAL(9,G44:G49)</f>
+      <c r="G60" s="131" t="n">
+        <f aca="false">SUBTOTAL(9,G43:G48)</f>
         <v>21</v>
       </c>
     </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <autoFilter ref="A2:H60">
     <sortState ref="A3:H60">

</xml_diff>